<commit_message>
Update README and add latest charts and report
</commit_message>
<xml_diff>
--- a/payments_quarterly_report.xlsx
+++ b/payments_quarterly_report.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +40,12 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -93,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -118,6 +124,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4859,7 +4866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5268,6 +5275,13 @@
       </c>
       <c r="I11" s="6" t="n">
         <v>117.41</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Note: This report covers all transaction types (domestic + cross-border). The boxplot chart filters to domestic transactions only for visual clarity. Both use the IQR method (beyond 1.5 × IQR from Q1/Q3).</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -5394,144 +5408,144 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Report Title</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="10" t="inlineStr">
         <is>
           <t>Euro Area Payments Statistics — Quarterly Series</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>Reference Period</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>2019-Q1 to 2024-Q4</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Generated</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>2026-07-13 23:08</t>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-14 13:15</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Data Source</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Synthetic data — Euro Area payments statistics framework</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Countries</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Country Coverage</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>20 euro area member states (EU countries using the EUR)</t>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Germany (DE) — largest euro area economy</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Instruments</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>card_payment, cheque, credit_transfer, direct_debit, e-money</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Total Rows</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>120</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>Outliers Flagged</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Outlier Flag</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>1 = statistically unusual observation, 0 = normal. Identified using z-score method per country and instrument series.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>Rounding Note</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Figures are stored at full precision and displayed rounded to 2 decimal places. Country-level totals in Country Indicators are rounded once after aggregation. Individual rows in Payments Statistics retain full precision — sums may therefore not add up exactly due to rounding, consistent with Euro Area statistical publication practice.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>YoY definition</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>% change vs same quarter one year prior (4 quarters back)</t>
         </is>

</xml_diff>